<commit_message>
Removed extra metadata column (peer review) from the summeries as it was earlier. Recalculated metrics.
</commit_message>
<xml_diff>
--- a/2_calculated_metrics/reference_corpus_metrics/reference_corpus_overview.xlsx
+++ b/2_calculated_metrics/reference_corpus_metrics/reference_corpus_overview.xlsx
@@ -12,36 +12,32 @@
     <sheet name="Journal Counts" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="All Feature Counts" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Source_Type" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Peer_Review" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Evidence_Type" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Primary_Methodology" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Evidence_Type" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Primary_Methodology" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Conceptual_Theme" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Library_Context" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Game_Format" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Service_Area" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Audience" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Service_Audience" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Intended_Outcome" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Evidence_Confidence" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Service_Conditions_Addressed" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Conceptual_Theme" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Coding_Confidence" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Year Counts'!$A$1:$C$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Journal Counts'!$A$1:$D$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All Feature Counts'!$A$1:$F$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All Feature Counts'!$A$1:$F$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Source_Type'!$A$1:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Peer_Review'!$A$1:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Evidence_Type'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Primary_Methodology'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Evidence_Type'!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Primary_Methodology'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Conceptual_Theme'!$A$1:$E$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Library_Context'!$A$1:$E$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Game_Format'!$A$1:$E$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Service_Area'!$A$1:$E$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Audience'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Service_Audience'!$A$1:$E$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Intended_Outcome'!$A$1:$E$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Evidence_Confidence'!$A$1:$E$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Service_Conditions_Addressed'!$A$1:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Conceptual_Theme'!$A$1:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Coding_Confidence'!$A$1:$E$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -462,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -537,7 +533,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9">
@@ -547,7 +543,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>76861</v>
+        <v>54312</v>
       </c>
     </row>
     <row r="10">
@@ -557,7 +553,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>10.674</v>
+        <v>7.542</v>
       </c>
     </row>
     <row r="11">
@@ -616,40 +612,40 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Peer_Review</t>
+          <t>Evidence_Type</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C16" t="n">
-        <v>7201</v>
+        <v>7223</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Evidence_Type</t>
+          <t>Primary_Methodology</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C17" t="n">
-        <v>7223</v>
+        <v>7201</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Primary_Methodology</t>
+          <t>Conceptual_Theme</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>7201</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -694,14 +690,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Audience</t>
+          <t>Service_Audience</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="C22" t="n">
-        <v>8147</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -741,32 +737,6 @@
       </c>
       <c r="C25" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Conceptual_Theme</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Coding_Confidence</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" t="n">
-        <v>7201</v>
       </c>
     </row>
   </sheetData>
@@ -1201,10 +1171,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -1238,217 +1208,9 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>5051</v>
-      </c>
-      <c r="C2" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D2" t="n">
-        <v>70.09999999999999</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>educators</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1472</v>
-      </c>
-      <c r="C3" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D3" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>students</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1048</v>
-      </c>
-      <c r="C4" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D4" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>general_public</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>183</v>
-      </c>
-      <c r="C5" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D5" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>children</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>112</v>
-      </c>
-      <c r="C6" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="E6" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>teens</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>105</v>
-      </c>
-      <c r="C7" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E7" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>underserved_or_special_population</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>52</v>
-      </c>
-      <c r="C8" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E8" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>adults</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>47</v>
-      </c>
-      <c r="C9" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E9" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>older_adults</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>40</v>
-      </c>
-      <c r="C10" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E10" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>families</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>21</v>
-      </c>
-      <c r="C11" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E11" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>young_adults</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>16</v>
-      </c>
-      <c r="C12" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E12" t="n">
-        <v>11</v>
-      </c>
-    </row>
+    <row r="2"/>
   </sheetData>
-  <autoFilter ref="A1:E12"/>
+  <autoFilter ref="A1:E2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1792,143 +1554,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>feature_value</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>article_count</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>total_articles</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>article_pct</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>rank_within_group</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-  </sheetData>
-  <autoFilter ref="A1:E2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>feature_value</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>article_count</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>total_articles</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>article_pct</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>rank_within_group</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>5322</v>
-      </c>
-      <c r="C2" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D2" t="n">
-        <v>73.90000000000001</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1879</v>
-      </c>
-      <c r="C3" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D3" t="n">
-        <v>26.1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2982,7 +2607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -3028,22 +2653,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>evidence_type</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>theoretical_or_conceptual</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5051</v>
+        <v>3729</v>
       </c>
       <c r="D2" t="n">
         <v>7201</v>
       </c>
       <c r="E2" t="n">
-        <v>70.09999999999999</v>
+        <v>51.8</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -3052,22 +2677,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>evidence_type</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>educators</t>
+          <t>empirical_study</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1472</v>
+        <v>2630</v>
       </c>
       <c r="D3" t="n">
         <v>7201</v>
       </c>
       <c r="E3" t="n">
-        <v>20.4</v>
+        <v>36.5</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
@@ -3076,22 +2701,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>evidence_type</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>students</t>
+          <t>implementation_case</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1048</v>
+        <v>292</v>
       </c>
       <c r="D4" t="n">
         <v>7201</v>
       </c>
       <c r="E4" t="n">
-        <v>14.6</v>
+        <v>4.1</v>
       </c>
       <c r="F4" t="n">
         <v>3</v>
@@ -3100,22 +2725,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>evidence_type</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>general_public</t>
+          <t>instrument_or_framework_development</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>183</v>
+        <v>253</v>
       </c>
       <c r="D5" t="n">
         <v>7201</v>
       </c>
       <c r="E5" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="F5" t="n">
         <v>4</v>
@@ -3124,22 +2749,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>evidence_type</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>children</t>
+          <t>evidence_synthesis</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>112</v>
+        <v>196</v>
       </c>
       <c r="D6" t="n">
         <v>7201</v>
       </c>
       <c r="E6" t="n">
-        <v>1.6</v>
+        <v>2.7</v>
       </c>
       <c r="F6" t="n">
         <v>5</v>
@@ -3148,22 +2773,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>evidence_type</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>teens</t>
+          <t>content_or_artifact_analysis</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="D7" t="n">
         <v>7201</v>
       </c>
       <c r="E7" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="F7" t="n">
         <v>6</v>
@@ -3172,190 +2797,190 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>underserved_or_special_population</t>
+          <t>unspecified_game_format</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>52</v>
+        <v>7160</v>
       </c>
       <c r="D8" t="n">
         <v>7201</v>
       </c>
       <c r="E8" t="n">
-        <v>0.7</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>adults</t>
+          <t>digital_game</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="D9" t="n">
         <v>7201</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>older_adults</t>
+          <t>virtual_or_augmented_reality</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="D10" t="n">
         <v>7201</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
       <c r="F10" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>families</t>
+          <t>gamification</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
         <v>7201</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>young_adults</t>
+          <t>tabletop_roleplaying_game</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
         <v>7201</v>
       </c>
       <c r="E12" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>coding_confidence</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>game_creation</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5322</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
         <v>7201</v>
       </c>
       <c r="E13" t="n">
-        <v>73.90000000000001</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>coding_confidence</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>escape_room_or_breakout_box</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1879</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
         <v>7201</v>
       </c>
       <c r="E14" t="n">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>evidence_type</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>theoretical_or_conceptual</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3729</v>
+        <v>3350</v>
       </c>
       <c r="D15" t="n">
         <v>7201</v>
       </c>
       <c r="E15" t="n">
-        <v>51.8</v>
+        <v>46.5</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
@@ -3364,22 +2989,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>evidence_type</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>empirical_study</t>
+          <t>learning_and_literacy</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2630</v>
+        <v>1496</v>
       </c>
       <c r="D16" t="n">
         <v>7201</v>
       </c>
       <c r="E16" t="n">
-        <v>36.5</v>
+        <v>20.8</v>
       </c>
       <c r="F16" t="n">
         <v>2</v>
@@ -3388,22 +3013,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>evidence_type</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>implementation_case</t>
+          <t>cultural_stewardship_and_preservation</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>292</v>
+        <v>930</v>
       </c>
       <c r="D17" t="n">
         <v>7201</v>
       </c>
       <c r="E17" t="n">
-        <v>4.1</v>
+        <v>12.9</v>
       </c>
       <c r="F17" t="n">
         <v>3</v>
@@ -3412,22 +3037,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>evidence_type</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>instrument_or_framework_development</t>
+          <t>creativity_and_production</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>253</v>
+        <v>713</v>
       </c>
       <c r="D18" t="n">
         <v>7201</v>
       </c>
       <c r="E18" t="n">
-        <v>3.5</v>
+        <v>9.9</v>
       </c>
       <c r="F18" t="n">
         <v>4</v>
@@ -3436,22 +3061,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>evidence_type</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>evidence_synthesis</t>
+          <t>institutional_capacity</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>196</v>
+        <v>709</v>
       </c>
       <c r="D19" t="n">
         <v>7201</v>
       </c>
       <c r="E19" t="n">
-        <v>2.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F19" t="n">
         <v>5</v>
@@ -3460,22 +3085,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>evidence_type</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>content_or_artifact_analysis</t>
+          <t>engagement_and_participation</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>123</v>
+        <v>607</v>
       </c>
       <c r="D20" t="n">
         <v>7201</v>
       </c>
       <c r="E20" t="n">
-        <v>1.7</v>
+        <v>8.4</v>
       </c>
       <c r="F20" t="n">
         <v>6</v>
@@ -3484,760 +3109,760 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>unspecified_game_format</t>
+          <t>discovery_and_advisory</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>7160</v>
+        <v>459</v>
       </c>
       <c r="D21" t="n">
         <v>7201</v>
       </c>
       <c r="E21" t="n">
-        <v>99.40000000000001</v>
+        <v>6.4</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>digital_game</t>
+          <t>belonging_and_community</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20</v>
+        <v>349</v>
       </c>
       <c r="D22" t="n">
         <v>7201</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3</v>
+        <v>4.8</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>virtual_or_augmented_reality</t>
+          <t>equitable_access</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>16</v>
+        <v>347</v>
       </c>
       <c r="D23" t="n">
         <v>7201</v>
       </c>
       <c r="E23" t="n">
-        <v>0.2</v>
+        <v>4.8</v>
       </c>
       <c r="F23" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>gamification</t>
+          <t>wellness_and_resilience</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>87</v>
       </c>
       <c r="D24" t="n">
         <v>7201</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="F24" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>tabletop_roleplaying_game</t>
+          <t>unspecified_library_context</t>
         </is>
       </c>
       <c r="C25" t="n">
+        <v>4839</v>
+      </c>
+      <c r="D25" t="n">
+        <v>7201</v>
+      </c>
+      <c r="E25" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="F25" t="n">
         <v>1</v>
-      </c>
-      <c r="D25" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>game_creation</t>
+          <t>academic_library</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>1639</v>
       </c>
       <c r="D26" t="n">
         <v>7201</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
       <c r="F26" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>escape_room_or_breakout_box</t>
+          <t>school_library</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>395</v>
       </c>
       <c r="D27" t="n">
         <v>7201</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="F27" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>cultural_heritage_institution</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3350</v>
+        <v>182</v>
       </c>
       <c r="D28" t="n">
         <v>7201</v>
       </c>
       <c r="E28" t="n">
-        <v>46.5</v>
+        <v>2.5</v>
       </c>
       <c r="F28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>learning_and_literacy</t>
+          <t>multiple_library_types</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1496</v>
+        <v>67</v>
       </c>
       <c r="D29" t="n">
         <v>7201</v>
       </c>
       <c r="E29" t="n">
-        <v>20.8</v>
+        <v>0.9</v>
       </c>
       <c r="F29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>cultural_stewardship_and_preservation</t>
+          <t>public_library</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>930</v>
+        <v>47</v>
       </c>
       <c r="D30" t="n">
         <v>7201</v>
       </c>
       <c r="E30" t="n">
-        <v>12.9</v>
+        <v>0.7</v>
       </c>
       <c r="F30" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>creativity_and_production</t>
+          <t>library_school</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>713</v>
+        <v>32</v>
       </c>
       <c r="D31" t="n">
         <v>7201</v>
       </c>
       <c r="E31" t="n">
-        <v>9.9</v>
+        <v>0.4</v>
       </c>
       <c r="F31" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>institutional_capacity</t>
+          <t>unspecified</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>709</v>
+        <v>5081</v>
       </c>
       <c r="D32" t="n">
         <v>7201</v>
       </c>
       <c r="E32" t="n">
-        <v>9.800000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="F32" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>engagement_and_participation</t>
+          <t>survey</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>607</v>
+        <v>636</v>
       </c>
       <c r="D33" t="n">
         <v>7201</v>
       </c>
       <c r="E33" t="n">
-        <v>8.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F33" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>discovery_and_advisory</t>
+          <t>qualitative_study</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>459</v>
+        <v>401</v>
       </c>
       <c r="D34" t="n">
         <v>7201</v>
       </c>
       <c r="E34" t="n">
-        <v>6.4</v>
+        <v>5.6</v>
       </c>
       <c r="F34" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>belonging_and_community</t>
+          <t>case_or_design_study</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>349</v>
+        <v>270</v>
       </c>
       <c r="D35" t="n">
         <v>7201</v>
       </c>
       <c r="E35" t="n">
-        <v>4.8</v>
+        <v>3.7</v>
       </c>
       <c r="F35" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>equitable_access</t>
+          <t>theoretical_or_conceptual</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>347</v>
+        <v>241</v>
       </c>
       <c r="D36" t="n">
         <v>7201</v>
       </c>
       <c r="E36" t="n">
-        <v>4.8</v>
+        <v>3.3</v>
       </c>
       <c r="F36" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>wellness_and_resilience</t>
+          <t>evidence_synthesis</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>87</v>
+        <v>196</v>
       </c>
       <c r="D37" t="n">
         <v>7201</v>
       </c>
       <c r="E37" t="n">
-        <v>1.2</v>
+        <v>2.7</v>
       </c>
       <c r="F37" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>unspecified_library_context</t>
+          <t>experimental_study</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>4839</v>
+        <v>174</v>
       </c>
       <c r="D38" t="n">
         <v>7201</v>
       </c>
       <c r="E38" t="n">
-        <v>67.2</v>
+        <v>2.4</v>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>academic_library</t>
+          <t>content_analysis</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1639</v>
+        <v>118</v>
       </c>
       <c r="D39" t="n">
         <v>7201</v>
       </c>
       <c r="E39" t="n">
-        <v>22.8</v>
+        <v>1.6</v>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>school_library</t>
+          <t>mixed_methods</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>395</v>
+        <v>57</v>
       </c>
       <c r="D40" t="n">
         <v>7201</v>
       </c>
       <c r="E40" t="n">
-        <v>5.5</v>
+        <v>0.8</v>
       </c>
       <c r="F40" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>cultural_heritage_institution</t>
+          <t>action_research</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>182</v>
+        <v>16</v>
       </c>
       <c r="D41" t="n">
         <v>7201</v>
       </c>
       <c r="E41" t="n">
-        <v>2.5</v>
+        <v>0.2</v>
       </c>
       <c r="F41" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>multiple_library_types</t>
+          <t>participatory_design</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>67</v>
+        <v>6</v>
       </c>
       <c r="D42" t="n">
         <v>7201</v>
       </c>
       <c r="E42" t="n">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="F42" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>public_library</t>
+          <t>historical_analysis</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="D43" t="n">
         <v>7201</v>
       </c>
       <c r="E43" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="F43" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>library_school</t>
+          <t>collections_and_access</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>32</v>
+        <v>2725</v>
       </c>
       <c r="D44" t="n">
         <v>7201</v>
       </c>
       <c r="E44" t="n">
-        <v>0.4</v>
+        <v>37.8</v>
       </c>
       <c r="F44" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>peer_review</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>peer_reviewed</t>
+          <t>discovery_and_advisory</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>7201</v>
+        <v>2056</v>
       </c>
       <c r="D45" t="n">
         <v>7201</v>
       </c>
       <c r="E45" t="n">
-        <v>100</v>
+        <v>28.6</v>
       </c>
       <c r="F45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>unspecified</t>
+          <t>learning_and_literacy</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>5081</v>
+        <v>1477</v>
       </c>
       <c r="D46" t="n">
         <v>7201</v>
       </c>
       <c r="E46" t="n">
-        <v>70.59999999999999</v>
+        <v>20.5</v>
       </c>
       <c r="F46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>survey</t>
+          <t>professional_capacity</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>636</v>
+        <v>862</v>
       </c>
       <c r="D47" t="n">
         <v>7201</v>
       </c>
       <c r="E47" t="n">
-        <v>8.800000000000001</v>
+        <v>12</v>
       </c>
       <c r="F47" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>qualitative_study</t>
+          <t>community_and_inclusion</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>401</v>
+        <v>676</v>
       </c>
       <c r="D48" t="n">
         <v>7201</v>
       </c>
       <c r="E48" t="n">
-        <v>5.6</v>
+        <v>9.4</v>
       </c>
       <c r="F48" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>case_or_design_study</t>
+          <t>programming_and_facilitation</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>270</v>
+        <v>411</v>
       </c>
       <c r="D49" t="n">
         <v>7201</v>
       </c>
       <c r="E49" t="n">
-        <v>3.7</v>
+        <v>5.7</v>
       </c>
       <c r="F49" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>theoretical_or_conceptual</t>
+          <t>creation_and_making</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>241</v>
+        <v>357</v>
       </c>
       <c r="D50" t="n">
         <v>7201</v>
       </c>
       <c r="E50" t="n">
-        <v>3.3</v>
+        <v>5</v>
       </c>
       <c r="F50" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>evidence_synthesis</t>
+          <t>outreach_and_partnerships</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>196</v>
+        <v>357</v>
       </c>
       <c r="D51" t="n">
         <v>7201</v>
       </c>
       <c r="E51" t="n">
-        <v>2.7</v>
+        <v>5</v>
       </c>
       <c r="F51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>experimental_study</t>
+          <t>cultural_heritage_and_research</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D52" t="n">
         <v>7201</v>
@@ -4246,395 +3871,59 @@
         <v>2.4</v>
       </c>
       <c r="F52" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>content_analysis</t>
+          <t>space_and_infrastructure</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>118</v>
+        <v>144</v>
       </c>
       <c r="D53" t="n">
         <v>7201</v>
       </c>
       <c r="E53" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="F53" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>source_type</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>mixed_methods</t>
+          <t>peer_reviewed_journal_article</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>57</v>
+        <v>7201</v>
       </c>
       <c r="D54" t="n">
         <v>7201</v>
       </c>
       <c r="E54" t="n">
-        <v>0.8</v>
+        <v>100</v>
       </c>
       <c r="F54" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>primary_methodology</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>action_research</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>16</v>
-      </c>
-      <c r="D55" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E55" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F55" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>primary_methodology</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>participatory_design</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>6</v>
-      </c>
-      <c r="D56" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E56" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F56" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>primary_methodology</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>historical_analysis</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>5</v>
-      </c>
-      <c r="D57" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E57" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F57" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>collections_and_access</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>2725</v>
-      </c>
-      <c r="D58" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E58" t="n">
-        <v>37.8</v>
-      </c>
-      <c r="F58" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>discovery_and_advisory</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
-        <v>2056</v>
-      </c>
-      <c r="D59" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E59" t="n">
-        <v>28.6</v>
-      </c>
-      <c r="F59" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>learning_and_literacy</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>1477</v>
-      </c>
-      <c r="D60" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E60" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="F60" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>professional_capacity</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>862</v>
-      </c>
-      <c r="D61" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E61" t="n">
-        <v>12</v>
-      </c>
-      <c r="F61" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>community_and_inclusion</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>676</v>
-      </c>
-      <c r="D62" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E62" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="F62" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>programming_and_facilitation</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>411</v>
-      </c>
-      <c r="D63" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E63" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="F63" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>creation_and_making</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>357</v>
-      </c>
-      <c r="D64" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E64" t="n">
-        <v>5</v>
-      </c>
-      <c r="F64" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>outreach_and_partnerships</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>357</v>
-      </c>
-      <c r="D65" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E65" t="n">
-        <v>5</v>
-      </c>
-      <c r="F65" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>cultural_heritage_and_research</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>173</v>
-      </c>
-      <c r="D66" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E66" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="F66" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>service_area</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>space_and_infrastructure</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>144</v>
-      </c>
-      <c r="D67" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E67" t="n">
-        <v>2</v>
-      </c>
-      <c r="F67" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>source_type</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>peer_reviewed_journal_article</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D68" t="n">
-        <v>7201</v>
-      </c>
-      <c r="E68" t="n">
-        <v>100</v>
-      </c>
-      <c r="F68" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F68"/>
+  <autoFilter ref="A1:F54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4713,74 +4002,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>feature_value</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>article_count</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>total_articles</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>article_pct</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>rank_within_group</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>peer_reviewed</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>7201</v>
-      </c>
-      <c r="C2" t="n">
-        <v>7201</v>
-      </c>
-      <c r="D2" t="n">
-        <v>100</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:E2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4938,7 +4159,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5211,6 +4432,56 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>feature_value</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>article_count</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>total_articles</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>article_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>rank_within_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>